<commit_message>
Inclui fotos do 2º Festival Fuzuê na prestação de contas da 27ª Parada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N6gWJWVRApAafkrjRjqz3P
</commit_message>
<xml_diff>
--- a/prestacao-contas-27-parada/Conferencia_Despesas_x_Fotos_27_Parada.xlsx
+++ b/prestacao-contas-27-parada/Conferencia_Despesas_x_Fotos_27_Parada.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conferência" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fotos da pasta" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fotos Fuzuê" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Conferência'!$A$1:$G$72</definedName>
@@ -2355,19 +2356,15 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>82</t>
-        </is>
-      </c>
-      <c r="F61" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>82, 83</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -2388,19 +2385,15 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>83</t>
-        </is>
-      </c>
-      <c r="F62" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G62" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>84, 85</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -2421,19 +2414,15 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>83</t>
-        </is>
-      </c>
-      <c r="F63" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>85, 86</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -2454,19 +2443,15 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="F64" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -2487,19 +2472,15 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>85</t>
-        </is>
-      </c>
-      <c r="F65" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -2520,19 +2501,15 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>85</t>
-        </is>
-      </c>
-      <c r="F66" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>83, 90</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -2553,19 +2530,15 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>85</t>
-        </is>
-      </c>
-      <c r="F67" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>89, 90</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -2586,7 +2559,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>91</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
@@ -2619,7 +2592,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>92</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
@@ -2652,19 +2625,15 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>87</t>
-        </is>
-      </c>
-      <c r="F70" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>93, 94, 95</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -2685,19 +2654,15 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>87</t>
-        </is>
-      </c>
-      <c r="F71" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G71" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>95, 96</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -2718,19 +2683,15 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>88</t>
-        </is>
-      </c>
-      <c r="F72" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>97, 98</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
@@ -3284,4 +3245,178 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Arquivos</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Conteúdo identificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>_DSC4141–4173</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Montagem: palco interno, fechamento, cenografia em tecido, backdrop CELLOS/Fuzuê, palco externo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>_DSC4174–4178</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Geradores com extintores</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>_DSC4179–4197</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Tendas (camarim/credenciamento, feira, apoio); PA do palco externo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>_DSC4198–4218</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Salas de apoio/camarim com mobiliário, área interna, equipe de produção</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>_DSC4219–4247</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Palco externo, cenografia (cisne, cactos), mesas e cadeiras da área de convivência</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>_DSC4248–4262</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Teste de luz, mesa de operação, kits/materiais</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>_DSC4263–4297</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bancadas/lounge, tendas de atendimento, segurança, ambulância, entrada com gradis</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>_DSC4298–4815</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Programação artística nos dois palcos (dança, drag, ballroom, shows, DJs) e público</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>_DSC4817</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mesma cena da montagem da Parada (_DSC4816) – provavelmente arquivo trocado de pasta</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C3589T01</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Fala institucional com banner da 27ª Parada (confirmar atividade)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C3590–C3617</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Montagem, credenciamento, geradores, controle de acesso com gradis</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C3618–C3706</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Apresentações, DJs no palco externo, público</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Inclui fotos das atividades conexas e da pasta de prestação de contas da Parada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N6gWJWVRApAafkrjRjqz3P
</commit_message>
<xml_diff>
--- a/prestacao-contas-27-parada/Conferencia_Despesas_x_Fotos_27_Parada.xlsx
+++ b/prestacao-contas-27-parada/Conferencia_Despesas_x_Fotos_27_Parada.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conferência" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fotos da pasta" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fotos Fuzuê" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fotos conexas e Parada #04" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Conferência'!$A$1:$G$72</definedName>
@@ -583,7 +584,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>73, 74</t>
+          <t>78, 79</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -616,7 +617,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -645,7 +646,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>20, 21, 22</t>
+          <t>22, 23, 24</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -674,7 +675,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>41</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -707,7 +708,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>28</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -736,7 +737,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>23, 24, 25</t>
+          <t>25, 26, 27</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -765,7 +766,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>11, 12, 13</t>
+          <t>12, 13, 14</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -794,7 +795,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>14, 15</t>
+          <t>15, 16</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -823,7 +824,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17, 18</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -852,7 +853,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>12, 17</t>
+          <t>13, 19</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -881,7 +882,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>37</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -914,7 +915,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>38</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -976,7 +977,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1096,7 +1097,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>27, 28</t>
+          <t>29, 30</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1125,7 +1126,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>39</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -1158,7 +1159,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>59</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1191,7 +1192,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>75</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -1224,7 +1225,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>31, 32</t>
+          <t>33, 34</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1282,7 +1283,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>92</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -1311,7 +1312,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>91</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1340,7 +1341,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>49</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -1373,7 +1374,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>47</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -1406,7 +1407,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>36</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -1435,7 +1436,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>36</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -1464,19 +1465,15 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>78</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>89, 90</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1526,7 +1523,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>57</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -1559,19 +1556,15 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>37</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -1592,7 +1585,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -1625,19 +1618,15 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>10, 42</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -1658,7 +1647,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>58</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -1691,7 +1680,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>58</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
@@ -1724,7 +1713,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>44</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
@@ -1786,7 +1775,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
@@ -1848,7 +1837,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>9, 10</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -1877,7 +1866,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>29, 30</t>
+          <t>31, 32</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -1906,7 +1895,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>22, 38</t>
+          <t>24, 40</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -1935,7 +1924,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>43</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
@@ -1968,7 +1957,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
@@ -1997,7 +1986,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>48</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
@@ -2030,19 +2019,15 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="F51" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>46, 56</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -2063,7 +2048,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>45</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
@@ -2092,19 +2077,15 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="F53" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -2125,19 +2106,15 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="F54" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -2158,7 +2135,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>85</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
@@ -2191,19 +2168,15 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="F56" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>83, 93</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -2224,19 +2197,15 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>81</t>
-        </is>
-      </c>
-      <c r="F57" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G57" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -2257,7 +2226,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>85</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
@@ -2290,19 +2259,15 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="F59" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G59" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -2323,19 +2288,15 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>76</t>
-        </is>
-      </c>
-      <c r="F60" s="5" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G60" s="2" t="inlineStr">
-        <is>
-          <t>Buscar foto com fotógrafo/equipe e inserir no espaço reservado</t>
-        </is>
-      </c>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -2356,7 +2317,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>82, 83</t>
+          <t>95, 96, 101</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -2385,7 +2346,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>84, 85</t>
+          <t>97, 98</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
@@ -2414,7 +2375,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>85, 86</t>
+          <t>98, 99</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
@@ -2443,7 +2404,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>100</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
@@ -2472,7 +2433,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>101, 102</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -2501,7 +2462,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>83, 90</t>
+          <t>96, 104</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
@@ -2530,7 +2491,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>89, 90</t>
+          <t>103, 104</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
@@ -2559,7 +2520,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>105</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
@@ -2592,7 +2553,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>106</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
@@ -2625,7 +2586,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>93, 94, 95</t>
+          <t>107, 108, 109</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
@@ -2654,7 +2615,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>95, 96</t>
+          <t>109, 110</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
@@ -2683,7 +2644,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>97, 98</t>
+          <t>111, 112</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
@@ -3253,7 +3214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3416,6 +3377,96 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Fuzuê #04</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Carga/descarga de estruturas, fechamentos, produção</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Pasta</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Conteúdo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Parada #04 Prestação de Contas (194)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cortejo e multidão (dia e noite), cordeiros, brigadistas com Bombeiros, climatizador, mesa de som, notebook, câmeras no trio, equipe credenciada, trios na dispersão</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Celebração 27 anos (147)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Prêmio Anyky Lima (cerimônia, homenageadas, público), painel de LED indoor, mobiliário, catering, troféus e disputa da BallRoom (House of Ve)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Encontro Mineiro de Paradas (16)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plenária na sede do CELLOS/MG, materiais institucionais</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Fotos LULA – Praça da Estação e Serraria (172)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>NÃO UTILIZADAS: registros de evento de campanha política ("Mulheres com Lula 13", "Área PCdoB"), não da Parada</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Marca octanorm como pendente de comprovação
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N6gWJWVRApAafkrjRjqz3P
</commit_message>
<xml_diff>
--- a/prestacao-contas-27-parada/Conferencia_Despesas_x_Fotos_27_Parada.xlsx
+++ b/prestacao-contas-27-parada/Conferencia_Despesas_x_Fotos_27_Parada.xlsx
@@ -1895,15 +1895,19 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>24, 40</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr"/>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Sem foto da Parada. Fotos da pasta "Fotos LULA" são de outro evento e não servem. Pedir ao fornecedor fotos do dia 19/07 + termo de entrega; se não foi montada, tratar como não executado.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">

</xml_diff>